<commit_message>
feat: agregar ejemplo de Estructuras de datos para el ciclo Ciclo-2026-Segundo-Semestre
</commit_message>
<xml_diff>
--- a/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/Video_Semana_5.xlsx
+++ b/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/Video_Semana_5.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardoajsivinac/Documents/GitHub/Cocosys/770-Introduccion-a-la-Programacion-y-Computacion-1/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08DE196A-9E9E-2D4E-AA9B-070F09014F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Video" sheetId="1" r:id="rId5"/>
+    <sheet name="Video" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -34,52 +43,75 @@
     <t>Link del Video</t>
   </si>
   <si>
-    <t>https://youtu.be/Z_deVzVUdnM</t>
-  </si>
-  <si>
     <t>**El video debe estar publicado en el canal de curso lo cual permite que sea accesible para todos los estudiantes y tutores</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8gzeeIbS8MA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
-    <font>
-      <sz val="10.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFF6D01"/>
       <name val="Arial"/>
-    </font>
-    <font>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font/>
-    <font>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
-    </font>
-    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF666666"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -88,7 +120,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -104,41 +136,54 @@
     </fill>
   </fills>
   <borders count="5">
-    <border/>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -148,55 +193,54 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -207,11 +251,17 @@
     <xdr:ext cx="704850" cy="962025"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="2" name="image1.png" title="Imagen">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -228,12 +278,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -423,114 +469,123 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="3" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+    </row>
+    <row r="2" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="8" t="s">
+      <c r="C5" s="11">
+        <v>5</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="10" t="s">
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="10"/>
+    </row>
+    <row r="8" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="10"/>
+    </row>
+    <row r="10" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B10" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="12" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C7"/>
-    <hyperlink r:id="rId2" ref="C8"/>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: agregar ejemplo de Estructuras de datos y contenido para el ciclo Ciclo-2026-Segundo-Semestre
</commit_message>
<xml_diff>
--- a/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/Video_Semana_5.xlsx
+++ b/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/Video_Semana_5.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardoajsivinac/Documents/GitHub/Sin título/Ciclo-2026-Segundo-Semestre/Contenido/5. Contenidos/Semana_5/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9C7C0E-8525-3A40-87F1-F5873AFE9B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Video" sheetId="1" r:id="rId5"/>
+    <sheet name="Video" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -34,51 +43,66 @@
     <t>Link del Video</t>
   </si>
   <si>
-    <t>https://youtu.be/Z_deVzVUdnM</t>
-  </si>
-  <si>
     <t>**El video debe estar publicado en el canal de curso lo cual permite que sea accesible para todos los estudiantes y tutores</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8gzeeIbS8MA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
-    <font>
-      <sz val="10.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFF6D01"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
-    <font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
-    </font>
-    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -88,7 +112,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -104,41 +128,54 @@
     </fill>
   </fills>
   <borders count="5">
-    <border/>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -148,55 +185,54 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -207,11 +243,17 @@
     <xdr:ext cx="704850" cy="962025"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="2" name="image1.png" title="Imagen">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -228,12 +270,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -423,114 +461,123 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="3" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+    </row>
+    <row r="2" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="8" t="s">
+      <c r="C5" s="11">
+        <v>5</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="10" t="s">
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="10"/>
+    </row>
+    <row r="8" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="10"/>
+    </row>
+    <row r="10" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B10" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="12" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C7"/>
-    <hyperlink r:id="rId2" ref="C8"/>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C8" r:id="rId2" xr:uid="{1FB9CB2D-8F3F-7340-A219-AAC63FCFD20C}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>